<commit_message>
feat: configure field mapping and source storage
</commit_message>
<xml_diff>
--- a/config/reference_tables.xlsx
+++ b/config/reference_tables.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,23 +463,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>B站</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
+          <t>小红书/抖音</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>#同花顺资讯</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>采访</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>新手教学</t>
-        </is>
-      </c>
+          <t>资讯</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>渠道固定规则</t>
+          <t>TAG权威映射</t>
         </is>
       </c>
     </row>
@@ -491,12 +491,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>#同花顺资讯</t>
+          <t>#同花顺股友说</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>资讯</t>
+          <t>股友说</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -514,12 +514,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>#同花顺股友说</t>
+          <t>#同顺图解</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>股友说</t>
+          <t>图文</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -537,12 +537,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>#同顺图解</t>
+          <t>#同顺盘点</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>图文</t>
+          <t>盘点</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -560,12 +560,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>#同顺盘点</t>
+          <t>#问财问句</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>盘点</t>
+          <t>问财</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -583,12 +583,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>#问财问句</t>
+          <t>#同顺深度财经</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>问财</t>
+          <t>长视频</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -606,12 +606,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>#同顺深度财经</t>
+          <t>#同顺财商</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>长视频</t>
+          <t>财商动画</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -629,39 +629,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>#同顺财商</t>
+          <t>#同花顺股民话题</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>财商动画</t>
+          <t>社区话题</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
-        <is>
-          <t>TAG权威映射</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>小红书/抖音</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>#同花顺股民话题</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>社区话题</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
         <is>
           <t>TAG权威映射</t>
         </is>
@@ -855,183 +832,600 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>来源文件</t>
+          <t>统一字段</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Sheet</t>
+          <t>标准字段</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>来源字段</t>
+          <t>字段角色</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>标准字段</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>字段角色</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>优先级</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>填充规则</t>
+          <t>Excel字段</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>*B站*</t>
+          <t>标题</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>sheet1</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Up主mid</t>
+          <t>identity</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>账号ID</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>账号</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>保留为账号ID，再通过账号映射表补实际账号名。</t>
+          <t>视频标题、标题、单元名称、创意名称、名称、计划名称、内容标题、笔记标题、链接、笔记/素材链接、__清洗行标题</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>*B站*</t>
+          <t>内容ID</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>sheet1</t>
+          <t>content_id</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>视频BVID</t>
+          <t>identity</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>视频/笔记id</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>标识</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>缺失时使用视频AVID。</t>
+          <t>视频BVID、视频bvid、视频id、视频ID、笔记ID、笔记/素材ID、广告ID、计划ID、内容ID、内容id、作品ID、id、ID、视频链接、链接、落地页、单元名称、__清洗行ID</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>*小红书*</t>
+          <t>备用内容ID</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>kos账户投放数据</t>
+          <t>content_id_fallback</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>发布作者</t>
+          <t>identity</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>实际账号</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>账号</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>小红书账号字段默认为实际账号名。</t>
+          <t>视频AVID</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>*抖音*</t>
+          <t>素材ID</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sheet2</t>
+          <t>material_id</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>账号/账号名称/发布账号/达人名称</t>
+          <t>identity</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>实际账号</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+          <t>素材ID、素材id、素材中心id、素材中心ID、计划ID、内容ID、视频id、笔记ID、链接、创意名称、单元名称、__清洗行ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>账号</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>抖音账号字段默认为实际账号名。</t>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>account</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>account</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>发布作者、账号、账号名称、发布账号、达人名称、Up主名称、UP主名称、UP主昵称、账户名称、作者</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>账号ID</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>account_id</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>account</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Up主mid、UID、uid、mid、账号ID、账号id、抖音号、达人ID、作者ID、用户ID、小红书号、账户ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>链接</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>content_url</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>链接、内容链接、视频链接、笔记链接、笔记/素材链接、素材url、落地页</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>封面</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>cover_url</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>视频封面图、封面、封面图、图片链接、素材url</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>时间</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>source_time</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>时间、日期、创建时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>时长</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>duration</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>时长</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>内容形式</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>content_form</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>内容类型</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>manual_category</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>内容分类、内容类型、内容类型_映射、__分组内容类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>消耗</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>spend</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>additive_metric</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>消耗、消费、花费、总花费、求和项:总花费、spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>曝光量</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>impressions</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>additive_metric</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>展示数、展示量、展现量、曝光次数、曝光量、曝光量(次)、视频展示量、求和项:展示量、impressions</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>点击量</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>clicks</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>additive_metric</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>点击量、点击数、点击次数、求和项:点击量、clicks</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>激活数</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>activations</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>additive_metric</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>激活数、激活数(转化时间)、应用激活数、APP激活数、APP激活次数、求和项:应用激活数、activations</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>付费数</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>first_pay_count</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>additive_metric</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>首次付费次数、首次付费次数(转化时间)、首次付费数、七日付费数、应用内付费、应用内首次付费次数、求和项:应用内首次付费次数、付费次数、付费数、注册次数、注册次数（点击归因）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>激活成本</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>activation_cost_raw</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>derived_metric_raw</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>激活成本、激活成本（元）、激活成本(转化时间)、应用激活成本、APP激活成本</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>付费成本</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>first_pay_cost_raw</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>derived_metric_raw</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>首次付费成本、首次付费成本(转化时间)、七日付费成本、应用内首次付费成本、付费成本、注册次数成本</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>点击率</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ctr_raw</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>derived_metric_raw</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>点击率</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>激活率</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>activation_rate_raw</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>derived_metric_raw</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>激活率、激活率%、激活率(转化时间)、应用激活率、APP点击激活率、APP下载激活率</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>付费率</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>first_pay_rate_raw</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>derived_metric_raw</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>首次付费率、首次付费率%、首次付费率(转化时间)、七日付费率、应用内首次付费率</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>点赞数</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>likes</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>点赞、点赞数、点赞量</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>评论数</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>comments</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>评论、评论量</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>收藏数</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>favorites</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>收藏</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>关注数</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>关注</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1103,49 +1497,15 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>一级分类</t>
+          <t>小红书/抖音TAG</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>不启用</t>
+          <t>TAG权威映射</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
-        <is>
-          <t>不区分长视频、短视频、图文；渠道就是第一层分析维度。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>B站栏目题材</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>采访 / 新手教学</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>B站不做动态栏目题材分类，统一按固定值写入。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>小红书/抖音TAG</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>TAG权威映射</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
         <is>
           <t>TAG命中时作为二级栏目来源，冲突进入人工审核。</t>
         </is>

</xml_diff>

<commit_message>
Prepare ops dashboard v1.5
</commit_message>
<xml_diff>
--- a/config/reference_tables.xlsx
+++ b/config/reference_tables.xlsx
@@ -22,16 +22,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,21 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,27 +422,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>渠道</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>标签词</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>二级栏目</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>三级题材</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>规则</t>
         </is>
@@ -659,27 +647,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>渠道</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>实际账号</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>二级栏目</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>三级题材</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
@@ -700,32 +688,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>渠道</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>来源账号ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>来源账号名</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>实际账号</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>映射来源</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
@@ -774,12 +762,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>段落</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>提示词</t>
         </is>
@@ -836,22 +824,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>统一字段</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>标准字段</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>字段角色</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Excel字段</t>
         </is>
@@ -1444,17 +1432,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>规则</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>取值</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>说明</t>
         </is>

</xml_diff>

<commit_message>
chore: preserve main wip before cleaning merge
</commit_message>
<xml_diff>
--- a/config/reference_tables.xlsx
+++ b/config/reference_tables.xlsx
@@ -22,13 +22,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,27 +434,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>渠道</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>标签词</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>二级栏目</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>三级题材</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>规则</t>
         </is>
@@ -647,27 +659,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>渠道</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>实际账号</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>二级栏目</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>三级题材</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
@@ -688,32 +700,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>渠道</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>来源账号ID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>来源账号名</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>实际账号</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>映射来源</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
@@ -762,12 +774,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>段落</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>提示词</t>
         </is>
@@ -824,22 +836,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>统一字段</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>标准字段</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>字段角色</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Excel字段</t>
         </is>
@@ -1215,7 +1227,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>首次付费次数、首次付费次数(转化时间)、首次付费数、七日付费数、应用内付费、应用内首次付费次数、求和项:应用内首次付费次数、付费次数、付费数、注册次数、注册次数（点击归因）</t>
+          <t>首次付费次数、首次付费次数(转化时间)、首次付费数、七日付费数、7日付费次数、应用内付费、应用内首次付费次数、求和项:应用内首次付费次数、付费次数、付费数、注册次数、注册次数（点击归因）</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1271,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>首次付费成本、首次付费成本(转化时间)、七日付费成本、应用内首次付费成本、付费成本、注册次数成本</t>
+          <t>首次付费成本、首次付费成本(转化时间)、七日付费成本、7日付费成本、应用内首次付费成本、付费成本、注册次数成本</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1337,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>首次付费率、首次付费率%、首次付费率(转化时间)、七日付费率、应用内首次付费率</t>
+          <t>首次付费率、首次付费率%、首次付费率(转化时间)、七日付费率、7日付费率、应用内首次付费率</t>
         </is>
       </c>
     </row>
@@ -1432,17 +1444,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>规则</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>取值</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>说明</t>
         </is>

</xml_diff>

<commit_message>
chore: preserve worktree wip before main merge
</commit_message>
<xml_diff>
--- a/config/reference_tables.xlsx
+++ b/config/reference_tables.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,6 +629,52 @@
       <c r="E9" t="inlineStr">
         <is>
           <t>TAG权威映射</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>B站市场部</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>采访</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>新手教学</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>渠道固定规则</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>B站商业化</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>采访</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>新手教学</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>渠道固定规则</t>
         </is>
       </c>
     </row>
@@ -684,7 +730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -722,7 +768,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>B站</t>
+          <t>B站市场部</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -742,6 +788,34 @@
         </is>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>B站导出账号为 Up主mid，已确认该 MID 对应同花顺投资。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B站商业化</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1622777305</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>同花顺投资</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>默认维护</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>B站导出账号为 Up主mid，已确认该 MID 对应同花顺投资。</t>
         </is>

</xml_diff>

<commit_message>
feat: stabilize ops recap workflow
</commit_message>
<xml_diff>
--- a/config/reference_tables.xlsx
+++ b/config/reference_tables.xlsx
@@ -22,13 +22,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,27 +434,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>渠道</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>标签词</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>二级栏目</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>三级题材</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>规则</t>
         </is>
@@ -693,27 +705,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>渠道</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>实际账号</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>二级栏目</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>三级题材</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
@@ -734,32 +746,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>渠道</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>来源账号ID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>来源账号名</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>实际账号</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>映射来源</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
@@ -836,12 +848,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>段落</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>提示词</t>
         </is>
@@ -898,22 +910,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>统一字段</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>标准字段</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>字段角色</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Excel字段</t>
         </is>
@@ -937,7 +949,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>视频标题、标题、单元名称、创意名称、名称、计划名称、内容标题、笔记标题、链接、笔记/素材链接、__清洗行标题</t>
+          <t>视频标题、标题、单元名称、创意名称、名称、计划名称、内容标题、笔记标题、笔记/素材名称、链接、笔记/素材链接、__清洗行标题</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1081,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>链接、内容链接、视频链接、笔记链接、笔记/素材链接、素材url、落地页</t>
+          <t>链接、内容链接、作品链接、视频链接、笔记链接、笔记/素材链接、素材url、落地页</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1191,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>内容分类、内容类型、内容类型_映射、__分组内容类型</t>
+          <t>内容分类、内容类型、二级、内容类型_映射、__分组内容类型</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1323,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>激活成本、激活成本（元）、激活成本(转化时间)、应用激活成本、APP激活成本</t>
+          <t>激活成本、激活成本（元）、激活成本(元)、激活成本(转化时间)、应用激活成本、APP激活成本</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1345,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>首次付费成本、首次付费成本(转化时间)、七日付费成本、7日付费成本、应用内首次付费成本、付费成本、注册次数成本</t>
+          <t>首次付费成本、首次付费成本(转化时间)、七日付费成本、7日付费成本、应用内首次付费成本、付费成本、付费成本(元)、注册次数成本</t>
         </is>
       </c>
     </row>
@@ -1506,17 +1518,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>规则</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>取值</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>说明</t>
         </is>

</xml_diff>

<commit_message>
feat: complete high value recap loop
</commit_message>
<xml_diff>
--- a/config/reference_tables.xlsx
+++ b/config/reference_tables.xlsx
@@ -906,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1110,144 +1110,144 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>时间</t>
+          <t>巨量链接</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>source_time</t>
+          <t>ad_material_url</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>context</t>
+          <t>evidence</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>时间、日期、创建时间</t>
+          <t>巨量素材链接、巨量链接、素材链接、素材url、素材URL、视频素材链接</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>时长</t>
+          <t>巨量封面链接</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>duration</t>
+          <t>ad_cover_url</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>context</t>
+          <t>evidence</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>时长</t>
+          <t>巨量封面链接、巨量封面、封面链接、视频封面图、封面图</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>内容形式</t>
+          <t>时间</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>content_form</t>
+          <t>source_time</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>context</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>类型</t>
+          <t>时间、日期、创建时间</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>内容类型</t>
+          <t>时长</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>manual_category</t>
+          <t>duration</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>context</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>内容分类、内容类型、二级、内容类型_映射、__分组内容类型</t>
+          <t>时长</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>消耗</t>
+          <t>内容形式</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>spend</t>
+          <t>content_form</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>additive_metric</t>
+          <t>content</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>消耗、消费、花费、总花费、求和项:总花费、spend</t>
+          <t>类型</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>曝光量</t>
+          <t>内容类型</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>impressions</t>
+          <t>manual_category</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>additive_metric</t>
+          <t>content</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>展示数、展示量、展现量、曝光次数、曝光量、曝光量(次)、视频展示量、求和项:展示量、impressions</t>
+          <t>内容分类、内容类型、二级、内容类型_映射、__分组内容类型</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>点击量</t>
+          <t>消耗</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>clicks</t>
+          <t>spend</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1257,19 +1257,19 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>点击量、点击数、点击次数、求和项:点击量、clicks</t>
+          <t>消耗、消费、花费、总花费、求和项:总花费、spend</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>激活数</t>
+          <t>曝光量</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>activations</t>
+          <t>impressions</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1279,19 +1279,19 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>激活数、激活数(转化时间)、应用激活数、APP激活数、APP激活次数、求和项:应用激活数、activations</t>
+          <t>展示数、展示量、展现量、曝光次数、曝光量、曝光量(次)、视频展示量、求和项:展示量、impressions</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>付费数</t>
+          <t>点击量</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>first_pay_count</t>
+          <t>clicks</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1301,63 +1301,63 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>首次付费次数、首次付费次数(转化时间)、首次付费数、七日付费数、7日付费次数、应用内付费、应用内首次付费次数、求和项:应用内首次付费次数、付费次数、付费数、注册次数、注册次数（点击归因）</t>
+          <t>点击量、点击数、点击次数、求和项:点击量、clicks</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>激活成本</t>
+          <t>激活数</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>activation_cost_raw</t>
+          <t>activations</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>derived_metric_raw</t>
+          <t>additive_metric</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>激活成本、激活成本（元）、激活成本(元)、激活成本(转化时间)、应用激活成本、APP激活成本</t>
+          <t>激活数、激活数(转化时间)、应用激活数、APP激活数、APP激活次数、求和项:应用激活数、activations</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>付费成本</t>
+          <t>付费数</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>first_pay_cost_raw</t>
+          <t>first_pay_count</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>derived_metric_raw</t>
+          <t>additive_metric</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>首次付费成本、首次付费成本(转化时间)、七日付费成本、7日付费成本、应用内首次付费成本、付费成本、付费成本(元)、注册次数成本</t>
+          <t>首次付费次数、首次付费次数(转化时间)、首次付费数、七日付费数、7日付费次数、应用内付费、应用内首次付费次数、求和项:应用内首次付费次数、付费次数、付费数、注册次数、注册次数（点击归因）</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>点击率</t>
+          <t>激活成本</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ctr_raw</t>
+          <t>activation_cost_raw</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1367,19 +1367,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>点击率</t>
+          <t>激活成本、激活成本（元）、激活成本(元)、激活成本(转化时间)、应用激活成本、APP激活成本</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>激活率</t>
+          <t>付费成本</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>activation_rate_raw</t>
+          <t>first_pay_cost_raw</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1389,19 +1389,19 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>激活率、激活率%、激活率(转化时间)、应用激活率、APP点击激活率、APP下载激活率</t>
+          <t>首次付费成本、首次付费成本(转化时间)、七日付费成本、7日付费成本、应用内首次付费成本、付费成本、付费成本(元)、注册次数成本</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>付费率</t>
+          <t>点击率</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>first_pay_rate_raw</t>
+          <t>ctr_raw</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1411,63 +1411,63 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>首次付费率、首次付费率%、首次付费率(转化时间)、七日付费率、7日付费率、应用内首次付费率</t>
+          <t>点击率</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>点赞数</t>
+          <t>激活率</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>activation_rate_raw</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>engagement</t>
+          <t>derived_metric_raw</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>点赞、点赞数、点赞量</t>
+          <t>激活率、激活率%、激活率(转化时间)、应用激活率、APP点击激活率、APP下载激活率</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>评论数</t>
+          <t>付费率</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>first_pay_rate_raw</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>engagement</t>
+          <t>derived_metric_raw</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>评论、评论量</t>
+          <t>首次付费率、首次付费率%、首次付费率(转化时间)、七日付费率、7日付费率、应用内首次付费率</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>收藏数</t>
+          <t>点赞数</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>favorites</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1477,27 +1477,71 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>收藏</t>
+          <t>点赞、点赞数、点赞量</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>评论数</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>comments</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>评论、评论量</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>收藏数</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>favorites</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>收藏</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>关注数</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>follows</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>engagement</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>关注</t>
         </is>

</xml_diff>